<commit_message>
Stage 7: define parametric specimen and fixture geometry
</commit_message>
<xml_diff>
--- a/literature/literature_matrix.xlsx
+++ b/literature/literature_matrix.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Literature" sheetId="1" r:id="R379c84a1a9474bff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="2" r:id="R64df492da6fd4de9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Literature" sheetId="1" r:id="R2a6ba552a3af4bd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="2" r:id="Rc6dd5e76555b4abb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -590,13 +590,13 @@
         <x:v>10.1016/j.addma.2022.102693</x:v>
       </x:c>
       <x:c r="G4" s="3" t="str">
-        <x:v>PLA; grade not extracted</x:v>
+        <x:v>Raise3D Premium PLA (§3.1)</x:v>
       </x:c>
       <x:c r="H4" s="3" t="str">
-        <x:v>Regular plate and bridge-like structure (Fig. 4)</x:v>
+        <x:v>Regular plate 60 × 10 × 4 mm and bridge-like structure 86 × 8 × 6 mm (Fig. 4)</x:v>
       </x:c>
       <x:c r="I4" s="3" t="str">
-        <x:v>Measured process histories; G-code-driven deposition</x:v>
+        <x:v>100% infill; 0.2 mm layer; 0.4 mm nozzle; 210 °C nozzle; 60 °C bed (§3.1)</x:v>
       </x:c>
       <x:c r="J4" s="3" t="str">
         <x:v>Printing thermal cycle; post-print annealing not the target</x:v>
@@ -2941,7 +2941,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R700056e2f5c147fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c35d84549b54c2c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3767,7 +3767,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62e43dccc2ed419a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71a3dc755da748f5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>